<commit_message>
Yucatán 2024: SFW's own Earth Connection photos as header, card and in-text pair; image export updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -19,8 +19,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-03 March 2025" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025-01 January 2025" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024-07 July 2024" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2023-08 August 2023" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2019-01 2019" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024-02 ERW February 2024" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2023-08 August 2023" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2019-01 2019" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -872,25 +873,21 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>No photos yet</t>
-        </is>
-      </c>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4204,6 +4201,262 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>2024-02 Ecosystem Restoration Workshop February 2024, Yucatán, México</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Images are final: cropped, colour-checked, max 1600 px (headers up to 2400 px), no EXIF data. Upload them as they are; do not crop them again in WordPress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>File name</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Where on the page</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Placement</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>How to show it</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Size (px)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Alt text</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Caption (gallery pop-up only)</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Photo credit</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>ecosystem-restoration-workshop-february-2024-header.jpg</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Header (top of page)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Top of the page, under the title</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Full content width, whole photo (no crop)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>2400 x 1793</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Three people walking along a red dirt track between green shrubs and trees, carrying buckets of seedlings, wide sun hats</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>From SFW's own 2023 registration page (promo.soilfoodweb.com/?p=106500); shows the reserve, not confirmed as taken during the workshop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>ecosystem-restoration-workshop-february-2024-card.jpg</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Workshops page card</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Card image on the Workshops listing page (/workshops/)</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>3:2 card, cut from the header photo</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>1200 x 800</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Three people walking along a red dirt track between green shrubs and trees, carrying buckets of seedlings, wide sun hats</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>ecosystem-restoration-workshop-february-2024-text-01.jpg</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>In the text</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>At the end of the section "What the workshop was for", photo 1 of 2 in the row</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Row of 2 photos side by side at the same height, whole photos</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>A person in a pink shirt and a straw hat bending to dig among dense green shrubs</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>From SFW's own 2023 registration page (promo.soilfoodweb.com/?p=106500); shows the reserve, not confirmed as taken during the workshop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>ecosystem-restoration-workshop-february-2024-text-02.jpg</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>In the text</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>At the end of the section "What the workshop was for", photo 2 of 2 in the row</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Row of 2 photos side by side at the same height, whole photos</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>960 x 720</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Looking up from the water of a cenote: tree roots hanging down the rock walls to the water, a wooden ladder, sunlight and trees at the opening</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>From SFW's own 2023 registration page (promo.soilfoodweb.com/?p=106500); shows the reserve, not confirmed as taken during the workshop.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5316,7 +5569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Remove the Brasil 2019 workshop: no evidence it officially took place
Page, card, Brasil filter and 2019 year option, past-workshop-images entry,
review listing and image export removed; the old URL redirects to
/workshops/. The photo file stays in the repo, unlinked.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -21,7 +21,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024-07 July 2024" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2024-02 ERW February 2024" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2023-08 August 2023" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2019-01 2019" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -949,36 +948,8 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>2019-01 Accelerator Workshop 2019, Brasil</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>https://finalsite-tau.vercel.app/workshops/accelerator-workshop-2019/</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Colours in the workshop sheets: yellow = header, purple = Workshops page card, blue = photo in the text, white = gallery.</t>
         </is>
@@ -5569,178 +5540,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>2019-01 Accelerator Workshop 2019, Brasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Images are final: cropped, colour-checked, max 1600 px (headers up to 2400 px), no EXIF data. Upload them as they are; do not crop them again in WordPress.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>File name</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Where on the page</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Placement</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>How to show it</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Size (px)</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Alt text</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Caption (gallery pop-up only)</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Photo credit</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>accelerator-workshop-2019-header.jpg</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Header (top of page)</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Top of the page, under the title</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Full content width, whole photo (no crop)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>444 x 188</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>A group of participants posing together indoors</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Low resolution (the only copy on file is 2025_08_brazil-2019.webp); replace with the original if found.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>accelerator-workshop-2019-card.jpg</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Workshops page card</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Card image on the Workshops listing page (/workshops/)</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>3:2 card, cut from the header photo</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>282 x 188</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>A group of participants posing together indoors</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="6" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Remove the México 2022 workshop: no evidence it officially took place
Page, card, 2022 year option, past-workshop-images entry, review listing
and export row removed; the old URL redirects to /workshops/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -916,40 +916,8 @@
       </c>
       <c r="H17" s="2" t="inlineStr"/>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>2022-03 Accelerator Workshop 2022, México</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>https://finalsite-tau.vercel.app/workshops/accelerator-workshop-2022/</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>No photos yet</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Colours in the workshop sheets: yellow = header, purple = Workshops page card, blue = photo in the text, white = gallery.</t>
         </is>

</xml_diff>

<commit_message>
India October 2026: header and card from the India registration page photos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -648,10 +648,10 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>1</v>
@@ -6042,7 +6042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>accelerator-workshop-october-2026-header.jpg</t>
+          <t>accelerator-workshop-october-2026-header-1.jpg</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -6139,22 +6139,22 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Top of the page, under the title</t>
+          <t>Left</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Full content width, whole photo (no crop)</t>
+          <t>Two photos side by side at the same height, together as one horizontal header</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>760 x 420</t>
+          <t>1080 x 1350</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>A collage: a compost tea brewer, a person at a microscope, a group of participants outdoors, hands holding compost, and the Accelerator Workshop logo</t>
+          <t>A woman in a green cap and gloves reaching into a tall pile of straw and hay inside a hoop house, others working behind her</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>
@@ -6162,42 +6162,156 @@
       <c r="J5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-october-2026-header-2.jpg</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Header (top of page)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Two photos side by side at the same height, together as one horizontal header</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>1080 x 1350</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>A room of students at long tables looking through microscopes, an instructor at a screen behind them</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-october-2026-header-3.jpg</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Header (top of page)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Two photos side by side at the same height, together as one horizontal header</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>1920 x 2400</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>A plate of South Indian food: vegetables, red rice, yellow rice, dal in steel bowls, peanuts and slices of watermelon</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-october-2026-header-4.jpg</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Header (top of page)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Two photos side by side at the same height, together as one horizontal header</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>1920 x 2400</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>A giant black statue of a face with a crescent moon, above a wide plaza with visitors, hills behind</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>accelerator-workshop-october-2026-card.jpg</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Workshops page card</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Card image on the Workshops listing page (/workshops/)</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>3:2 card, cut from the header photo</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>630 x 420</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>A collage: a compost tea brewer, a person at a microscope, a group of participants outdoors, hands holding compost, and the Accelerator Workshop logo</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>1200 x 800</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>A giant black statue of a face with a crescent moon on its head, against a pale sky</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
India October 2026 header: venue photos only from the registration page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -6149,12 +6149,12 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>1080 x 1350</t>
+          <t>1920 x 2400</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>A woman in a green cap and gloves reaching into a tall pile of straw and hay inside a hoop house, others working behind her</t>
+          <t>A giant black statue of a face with a crescent moon, above a wide plaza with visitors, hills behind</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>
@@ -6187,12 +6187,12 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>1080 x 1350</t>
+          <t>1920 x 2400</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>A room of students at long tables looking through microscopes, an instructor at a screen behind them</t>
+          <t>People bathing in a large stone-walled pool under a tiled roof, a red curtain on one side</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr"/>
@@ -6268,7 +6268,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>A giant black statue of a face with a crescent moon, above a wide plaza with visitors, hills behind</t>
+          <t>A simple room with two low beds, an orange wall, a white door and a tall white cupboard</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Past workshop pages: final texts word for word (13 October); WordPress downloads: new photo spots and the 16 new June 2025 gallery photos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -510,6 +510,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -760,7 +761,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="D12" s="2" t="n">
         <v>1</v>
@@ -772,7 +773,7 @@
         <v>3</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
     </row>
@@ -916,6 +917,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr"/>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -1107,7 +1109,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "Where students learned", photo 1 of 2 in the row</t>
+          <t>After paragraph 1 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1145,7 +1147,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "Where students learned", photo 2 of 2 in the row</t>
+          <t>After paragraph 1 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1183,7 +1185,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students did", photo 1 of 2 in the row</t>
+          <t>After paragraph 2 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -1221,7 +1223,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students did", photo 2 of 2 in the row</t>
+          <t>After paragraph 2 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -1259,7 +1261,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students said", photo 1 of 2 in the row</t>
+          <t>After paragraph 4 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1297,7 +1299,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students said", photo 2 of 2 in the row</t>
+          <t>After paragraph 4 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -2553,7 +2555,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", on its own</t>
+          <t>After paragraph 2 of the text</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -2759,7 +2761,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 1 of 4 in the row</t>
+          <t>After paragraph 2 of the text, photo 1 of 4 in the row</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -2797,7 +2799,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 2 of 4 in the row</t>
+          <t>After paragraph 2 of the text, photo 2 of 4 in the row</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -2835,7 +2837,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 3 of 4 in the row</t>
+          <t>After paragraph 2 of the text, photo 3 of 4 in the row</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -2873,7 +2875,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 4 of 4 in the row</t>
+          <t>After paragraph 2 of the text, photo 4 of 4 in the row</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -4317,7 +4319,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 1 of 2 in the row</t>
+          <t>After paragraph 2 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -4359,7 +4361,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 2 of 2 in the row</t>
+          <t>After paragraph 2 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -4569,7 +4571,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 1 of 2 in the row</t>
+          <t>After paragraph 1 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -4607,7 +4609,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 2 of 2 in the row</t>
+          <t>After paragraph 1 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -4645,7 +4647,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "Why it matters", photo 1 of 2 in the row</t>
+          <t>After paragraph 3 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -4683,7 +4685,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "Why it matters", photo 2 of 2 in the row</t>
+          <t>After paragraph 3 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -6703,7 +6705,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students did", photo 1 of 2 in the row</t>
+          <t>After paragraph 1 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -6741,7 +6743,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students did", photo 2 of 2 in the row</t>
+          <t>After paragraph 1 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -6779,7 +6781,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "The first workshop without Dr. Elaine", photo 1 of 2 in the row</t>
+          <t>After paragraph 3 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -6817,7 +6819,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "The first workshop without Dr. Elaine", photo 2 of 2 in the row</t>
+          <t>After paragraph 3 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -7947,7 +7949,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students did", on its own</t>
+          <t>After paragraph 2 of the text</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -9030,7 +9032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9059,6 +9061,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -9203,7 +9206,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 1 of 2 in the row</t>
+          <t>After paragraph 2 of the text, photo 1 of 2 in the row</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -9241,7 +9244,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What the workshop was for", photo 2 of 2 in the row</t>
+          <t>After paragraph 2 of the text, photo 2 of 2 in the row</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -9279,7 +9282,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>At the end of the section "What students did", on its own</t>
+          <t>After paragraph 4 of the text</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -9317,7 +9320,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Photo 1 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 1 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -9359,7 +9362,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Photo 2 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 2 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -9401,7 +9404,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Photo 3 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 3 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -9443,7 +9446,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Photo 4 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 4 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -9485,7 +9488,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Photo 5 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 5 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -9527,7 +9530,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Photo 6 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 6 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -9569,7 +9572,7 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Photo 7 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 7 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -9611,7 +9614,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Photo 8 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 8 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -9653,7 +9656,7 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Photo 9 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 9 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -9695,7 +9698,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Photo 10 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 10 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -9737,7 +9740,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Photo 11 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 11 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -9779,7 +9782,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Photo 12 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 12 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -9821,7 +9824,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Photo 13 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 13 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -9863,7 +9866,7 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Photo 14 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 14 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -9905,7 +9908,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Photo 15 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 15 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -9947,7 +9950,7 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Photo 16 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 16 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -9989,7 +9992,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Photo 17 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 17 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -10031,7 +10034,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Photo 18 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 18 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -10073,7 +10076,7 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Photo 19 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 19 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -10115,7 +10118,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Photo 20 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 20 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -10157,7 +10160,7 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Photo 21 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 21 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -10199,7 +10202,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Photo 22 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 22 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -10241,7 +10244,7 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Photo 23 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 23 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -10283,7 +10286,7 @@
       </c>
       <c r="D33" s="8" t="inlineStr">
         <is>
-          <t>Photo 24 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 24 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -10325,7 +10328,7 @@
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>Photo 25 of 25, under the heading "Photos from the workshop"</t>
+          <t>Photo 25 of 41, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -10350,6 +10353,678 @@
       </c>
       <c r="I34" s="8" t="inlineStr"/>
       <c r="J34" s="8" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-26-compost-build-green-material.jpg</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Photo 26 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Four people in hats and gloves watering and forking a large pile of fresh green material on a blue tarp in the barn</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Building a pile with fresh green material</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="n"/>
+      <c r="J35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-27-soil-sampling-in-the-meadow.jpg</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Photo 27 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Participants with clipboards gathered around a man kneeling at a soil sample in a grassy meadow with poppies, a farmhouse behind</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Soil sampling in the meadow</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="n"/>
+      <c r="J36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-28-morning-over-the-fields.jpg</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Photo 28 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 721</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>A field tinged red with poppies, red-roofed farm buildings and woodland under a clear blue sky</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Morning over the Wild Ken Hill fields</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="n"/>
+      <c r="J37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-29-lifting-the-cage.jpg</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Photo 29 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 721</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Participants in the barn entrance around two cylinders of compost, one just lifted out of its wire cage</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>Lifting the cage off a finished pile</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="n"/>
+      <c r="J38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-30-beside-the-windrow-turner.jpg</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Photo 30 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>A smiling woman in a cap and denim apron stands in a green field beside a long compost windrow, a tractor, water tanker and windrow turner behind</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>Beside the windrow turner</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="n"/>
+      <c r="J39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-31-poppies-in-bloom.jpg</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Photo 31 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 720</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>A dense field of bright red poppies in front of a dark treeline</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Poppies in bloom</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="n"/>
+      <c r="J40" s="8" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-32-evening-on-the-beach.jpg</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Photo 32 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 720</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Participants sitting in a loose circle on a sandy beach at dusk, dune grass behind and the sea on the horizon</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>Evening on the beach</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-33-morning-on-the-beach.jpg</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Photo 33 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Two smiling women in the foreground, the group sitting on the sand behind them with snacks, sea and dunes</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>A morning on the beach</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-34-walking-out-to-the-fields.jpg</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Photo 34 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 721</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>The group walking single file along a grassy track toward a field with red poppies</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Walking out to the fields</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-35-under-the-oaks.jpg</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Photo 35 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>The group standing along a dirt farm track under large oak trees, blue sky with white clouds</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>Under the oaks on the farm track</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-36-talking-it-through.jpg</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Photo 36 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Participants in grey t-shirts and wellies laughing with an older man in a blue polo on a grassy track, trees behind</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>Talking it through after the walk</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="n"/>
+      <c r="J45" s="8" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-37-pizza-van-lunch.jpg</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Photo 37 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 720</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Participants queuing at a red and cream vintage van serving wood-fired pizza, brick barns behind</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Wood-fired pizza for lunch</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="n"/>
+      <c r="J46" s="8" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-38-a-finished-pile.jpg</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Photo 38 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>The group cheering with arms raised around a finished wire-caged compost pile in the barn</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>A finished pile</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="n"/>
+      <c r="J47" s="8" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-39-evening-at-the-farm.jpg</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Photo 39 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1204</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Participants relaxing at picnic tables on the grass beside farm sheds under an evening sky</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Evening at the farm</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="n"/>
+      <c r="J48" s="8" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-40-into-the-woodland.jpg</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Photo 40 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Participants walking single file along a narrow path through tall green grass in woodland</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>Into the rewilded woodland</t>
+        </is>
+      </c>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2025-gallery-41-through-the-bracken.jpg</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Photo 41 of 41, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Participants pushing through head-high green bracken ferns in woodland, seen from behind</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Through the bracken</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
June 2026 Wild Ken Hill: 20-photo gallery from the June 2026 SFW Drive folder; download, spreadsheets and image catalog updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPK2bWpBHPAitKEehw7gcL
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -116,6 +116,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -677,7 +680,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>2</v>
@@ -689,7 +692,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
     </row>
@@ -6326,7 +6329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6355,6 +6358,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -6520,6 +6524,846 @@
       <c r="H7" s="6" t="inlineStr"/>
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-01-morning-lecture.jpg</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Photo 1 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Participants seated at white tables in a barn classroom, facing two screens and a whiteboard</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Day one in the barn classroom</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-02-pressed-leaves.jpg</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Photo 2 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Hands holding an open notebook of pressed leaves over a heap of fresh green feedstock</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Matching leaves to the green feedstock</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="n"/>
+      <c r="J9" s="9" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-03-class-circle.jpg</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Photo 3 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>The class standing in a circle on the grass around a heap of green feedstock, picnic tables and fields behind</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>Gathering round the first feedstock</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-04-checking-compost.jpg</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Photo 4 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>People bending over a heap of compost on a blue tarp, one holding a yellow clipboard</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>A close look at the compost</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-05-hands-in-compost.jpg</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Photo 5 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>A woman in gloves kneeling to work dark compost on a blue tarp</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>Hands in the compost</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-06-layered-feedstock.jpg</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Photo 6 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>Layers of feedstock on a blue tarp: yellow grain, grey wool and green plant material</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Layering up a pile recipe</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-07-team-at-the-bin.jpg</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Photo 7 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>1600 x 747</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Five people laughing and leaning on a filled wire compost bin in the barn, black buckets stacked beside it</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>A team with their new pile</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-08-bucket-of-compost.jpg</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Photo 8 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>A smiling man in overalls holding a black bucket of dark compost outside the barn, a field behind</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>A bucket of the good stuff</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="n"/>
+      <c r="J15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-09-watering-the-pile.jpg</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Photo 9 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>901 x 1600</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>A woman in a red top and blue apron watering a filled wire compost bin in the barn, others watching</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Watering in a fresh pile</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-10-inside-the-bin.jpg</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Photo 10 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>A person in a blue hat and pink gloves standing inside a round mesh compost bin, a smiling woman holding the rim</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Climbing in to level the pile</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="9" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-11-field-session.jpg</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Photo 11 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>A woman in a red shirt and visor sitting in the grass explaining a sampling kit, a man sitting beside her</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>A field session in the grass</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="n"/>
+      <c r="J18" s="9" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-12-thermometer-in-the-grass.jpg</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Photo 12 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>A compost thermometer dial lying in the grass among small purple wildflowers</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>A thermometer resting among the wildflowers</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="n"/>
+      <c r="J19" s="9" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-13-farmyard.jpg</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Photo 13 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>The class gathered by a tractor and a large water tank in a farmyard, barns behind, blue sky</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>Out in the farmyard</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="n"/>
+      <c r="J20" s="9" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-14-talking-it-over.jpg</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Photo 14 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Two men in caps talking over a steel grid, blue sky behind</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Talking it over</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="n"/>
+      <c r="J21" s="9" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-15-turner-paddles.jpg</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Photo 15 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>The steel paddles of a windrow turner coated in compost, a tractor and a man in a blue shirt below, clear blue sky</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>The windrow turner up close</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-16-windrow.jpg</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Photo 16 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>A man in a blue shirt bending over a dark compost windrow in a field, three people in caps behind</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Checking the windrow in the field</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="n"/>
+      <c r="J23" s="9" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-17-field-with-poppies.jpg</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Photo 17 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>The group standing in a field with poppies at the edge, many in sun hats, hedges and blue sky</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>A field day among the poppies</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="n"/>
+      <c r="J24" s="9" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-18-spray-bottles.jpg</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Photo 18 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>A woman in a straw hat holding two green spray bottles in a field</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>Ready to spray</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="n"/>
+      <c r="J25" s="9" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-19-beach-sunset.jpg</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Photo 19 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>A man sitting on a beach at sunset holding a piece of driftwood, a small fire bowl beside him, the sea behind</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Sunset on the beach</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="n"/>
+      <c r="J26" s="9" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-june-2026-gallery-20-campfire.jpg</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Photo 20 of 20, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>People sitting around a campfire on the beach at night, faces lit by the flames</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Around the fire on the last nights</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="n"/>
+      <c r="J27" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9061,7 +9905,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
February 2026 Santa Fe: 20 more gallery photos from Photos-Feb26-CTPAW (42 in total); download, spreadsheets, image log and catalog updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012wRfeXMPTbC6eXZxZinR6X
</commit_message>
<xml_diff>
--- a/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
+++ b/exports/workshop-images/workshop-images-for-wordpress-all-workshops.xlsx
@@ -513,7 +513,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -708,7 +707,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>1</v>
@@ -720,7 +719,7 @@
         <v>4</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
     </row>
@@ -6358,7 +6357,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -7376,7 +7374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7701,7 +7699,7 @@
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>Photo 1 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 1 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -7724,16 +7722,16 @@
           <t>Synergia Ranch, our home for the two weeks</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr"/>
-      <c r="J11" s="8" t="inlineStr"/>
-    </row>
-    <row r="12">
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="8" t="n"/>
+    </row>
+    <row r="12" ht="79.25" customHeight="1">
       <c r="A12" s="8" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-02-baby-goat.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-02-cholla.jpg</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -7743,7 +7741,7 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Photo 2 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 2 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -7753,29 +7751,33 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>1600 x 900</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>A baby goat lying in dry grass next to a sheep</t>
+          <t>Cholla cactus with small yellow fruit in dry grass, hills and blue sky behind</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>A new friend at the ranch</t>
-        </is>
-      </c>
-      <c r="I12" s="8" t="inlineStr"/>
-      <c r="J12" s="8" t="inlineStr"/>
-    </row>
-    <row r="13">
+          <t>Cholla cactus on the ranch</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="n"/>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="79.25" customHeight="1">
       <c r="A13" s="8" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-03-classroom.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-03-windrow-in-the-desert.jpg</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
@@ -7785,7 +7787,7 @@
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>Photo 3 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 3 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -7795,29 +7797,33 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>1600 x 900</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>A full classroom seen from the back: long tables, a wooden beam ceiling and many students with laptops</t>
+          <t>A long compost windrow on dry ground, bare trees, juniper and blue mountains behind</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>A full classroom</t>
-        </is>
-      </c>
-      <c r="I13" s="8" t="inlineStr"/>
-      <c r="J13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14">
+          <t>A windrow in the high desert</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="79.25" customHeight="1">
       <c r="A14" s="8" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-04-instructor-at-whiteboard.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-04-wagon-wheels.jpg</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -7827,7 +7833,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Photo 4 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 4 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -7837,21 +7843,25 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>1600 x 1200</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>An instructor in a plaid shirt speaking into a microphone in front of a whiteboard</t>
+          <t>Old wooden wagon wheels lying in dry grass under bare trees</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>Class in session</t>
-        </is>
-      </c>
-      <c r="I14" s="8" t="inlineStr"/>
-      <c r="J14" s="8" t="inlineStr"/>
+          <t>Old wagon wheels in the scrub</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
@@ -7859,7 +7869,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-05-instructor-outdoors.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-05-baby-goat.jpg</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -7869,7 +7879,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Photo 5 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 5 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -7879,29 +7889,29 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>900 x 1600</t>
+          <t>1600 x 900</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>An instructor in a rust fleece speaking outdoors, with a shed and a hoop house behind him</t>
+          <t>A baby goat lying in dry grass next to a sheep</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>Teaching outdoors</t>
-        </is>
-      </c>
-      <c r="I15" s="8" t="inlineStr"/>
-      <c r="J15" s="8" t="inlineStr"/>
-    </row>
-    <row r="16">
+          <t>A new friend at the ranch</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="8" t="n"/>
+    </row>
+    <row r="16" ht="79.25" customHeight="1">
       <c r="A16" s="8" t="n">
         <v>12</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-06-class-walking.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-06-flower-tiles.jpg</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -7911,7 +7921,7 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Photo 6 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 6 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -7921,21 +7931,25 @@
       </c>
       <c r="F16" s="8" t="inlineStr">
         <is>
-          <t>1600 x 1200</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>The class walking in a line along a dirt path through dry scrub</t>
+          <t>Wall tiles painted with yellow flowers between rows of green tiles</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>Off on a walk across the ranch</t>
-        </is>
-      </c>
-      <c r="I16" s="8" t="inlineStr"/>
-      <c r="J16" s="8" t="inlineStr"/>
+          <t>Yellow flower tiles</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -7943,7 +7957,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-07-inspecting-feedstock.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-07-classroom.jpg</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -7953,7 +7967,7 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>Photo 7 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 7 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -7968,16 +7982,16 @@
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>A woman in a red jacket reaching into a blue drum of dry feedstock, with students in green caps around her</t>
+          <t>A full classroom seen from the back: long tables, a wooden beam ceiling and many students with laptops</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>Getting hands-on with feedstock</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr"/>
-      <c r="J17" s="8" t="inlineStr"/>
+          <t>A full classroom</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -7985,7 +7999,7 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-08-students-at-feedstock-drums.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-08-instructor-at-whiteboard.jpg</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -7995,7 +8009,7 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Photo 8 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 8 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -8005,29 +8019,29 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>900 x 1100</t>
+          <t>1600 x 1200</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Students crouched and kneeling at blue drums of feedstock, with shade structures behind</t>
+          <t>An instructor in a plaid shirt speaking into a microphone in front of a whiteboard</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>Inspecting feedstock together</t>
-        </is>
-      </c>
-      <c r="I18" s="8" t="inlineStr"/>
-      <c r="J18" s="8" t="inlineStr"/>
-    </row>
-    <row r="19">
+          <t>Class in session</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="n"/>
+      <c r="J18" s="8" t="n"/>
+    </row>
+    <row r="19" ht="79.25" customHeight="1">
       <c r="A19" s="8" t="n">
         <v>15</v>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-09-feedstock-from-above.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-09-comparing-notes.jpg</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -8037,7 +8051,7 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>Photo 9 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 9 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -8047,29 +8061,33 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>1600 x 900</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Blue drums of dry stems seen from above, a hand reaching in and a person in a straw hat</t>
+          <t>A bearded man in a green cap and a woman looking at something in his hands in the classroom, students at laptops behind</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>Feedstock, up close</t>
-        </is>
-      </c>
-      <c r="I19" s="8" t="inlineStr"/>
-      <c r="J19" s="8" t="inlineStr"/>
-    </row>
-    <row r="20">
+          <t>Comparing notes in the classroom</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="79.25" customHeight="1">
       <c r="A20" s="8" t="n">
         <v>16</v>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-10-aged-wood-chips.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-10-sample-to-the-light.jpg</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
@@ -8079,7 +8097,7 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Photo 10 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 10 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -8089,21 +8107,25 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>1600 x 1200</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>A pile of aged wood chips with a blue label reading "Aged wood chips"</t>
+          <t>A woman in a plaid shirt and name tag holding up a pipette and a sample tube in the classroom, a projector screen behind</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>Aged wood chips, ready for the pile</t>
-        </is>
-      </c>
-      <c r="I20" s="8" t="inlineStr"/>
-      <c r="J20" s="8" t="inlineStr"/>
+          <t>A sample, held up to the light</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
@@ -8111,7 +8133,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-11-alfalfa-cubes.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-11-instructor-outdoors.jpg</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -8121,7 +8143,7 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>Photo 11 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 11 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -8131,21 +8153,21 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>1600 x 1200</t>
+          <t>900 x 1600</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>A sack labeled "Alfalfa Cubes, net wt. 50 lb"</t>
+          <t>An instructor in a rust fleece speaking outdoors, with a shed and a hoop house behind him</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>Alfalfa cubes for the compost recipe</t>
-        </is>
-      </c>
-      <c r="I21" s="8" t="inlineStr"/>
-      <c r="J21" s="8" t="inlineStr"/>
+          <t>Teaching outdoors</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="n"/>
+      <c r="J21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -8153,7 +8175,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-12-feedstock-buckets.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-12-class-walking.jpg</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -8163,7 +8185,7 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Photo 12 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 12 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -8173,29 +8195,29 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>1600 x 900</t>
+          <t>1600 x 1200</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>Rows of blue buckets of dark feedstock, with a hoop house and a hill behind</t>
+          <t>The class walking in a line along a dirt path through dry scrub</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>Feedstocks lined up for pile building</t>
-        </is>
-      </c>
-      <c r="I22" s="8" t="inlineStr"/>
-      <c r="J22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23">
+          <t>Off on a walk across the ranch</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="n"/>
+      <c r="J22" s="8" t="n"/>
+    </row>
+    <row r="23" ht="79.25" customHeight="1">
       <c r="A23" s="8" t="n">
         <v>19</v>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-13-thermometer-in-hay-bale.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-13-by-the-hoop-houses.jpg</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -8205,7 +8227,7 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Photo 13 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 13 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -8215,21 +8237,25 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>1200 x 1600</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>A long-stem compost thermometer and a sun hat on a hay bale</t>
+          <t>Three men smiling in front of a row of shade-cloth hoop houses, a blue tarp and pallets beside them, clear blue sky</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>The compost thermometer, always close at hand</t>
-        </is>
-      </c>
-      <c r="I23" s="8" t="inlineStr"/>
-      <c r="J23" s="8" t="inlineStr"/>
+          <t>By the hoop houses</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="n"/>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
@@ -8237,7 +8263,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-14-class-in-hoop-house.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-14-inspecting-feedstock.jpg</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -8247,7 +8273,7 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Photo 14 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 14 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -8257,21 +8283,21 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>1600 x 1200</t>
+          <t>1600 x 900</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Students in caps and wide hats standing close together inside a hoop house, listening</t>
+          <t>A woman in a red jacket reaching into a blue drum of dry feedstock, with students in green caps around her</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>Listening in the hoop house</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr"/>
-      <c r="J24" s="8" t="inlineStr"/>
+          <t>Getting hands-on with feedstock</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
@@ -8279,7 +8305,7 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-15-insulated-compost-pile.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-15-students-at-feedstock-drums.jpg</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
@@ -8289,7 +8315,7 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>Photo 15 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 15 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -8299,21 +8325,21 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>1200 x 1600</t>
+          <t>900 x 1100</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>A woody compost pile in a hoop house, its base wrapped in reflective insulation</t>
+          <t>Students crouched and kneeling at blue drums of feedstock, with shade structures behind</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>A pile wrapped up against the winter cold</t>
-        </is>
-      </c>
-      <c r="I25" s="8" t="inlineStr"/>
-      <c r="J25" s="8" t="inlineStr"/>
+          <t>Inspecting feedstock together</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
@@ -8321,7 +8347,7 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-16-compost-row-in-hoop-house.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-16-feedstock-from-above.jpg</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -8331,7 +8357,7 @@
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Photo 16 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 16 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -8341,21 +8367,21 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>1200 x 1600</t>
+          <t>1600 x 900</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>The inside of a hoop house with a long row of dark compost</t>
+          <t>Blue drums of dry stems seen from above, a hand reaching in and a person in a straw hat</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>A long row of compost in the hoop house</t>
-        </is>
-      </c>
-      <c r="I26" s="8" t="inlineStr"/>
-      <c r="J26" s="8" t="inlineStr"/>
+          <t>Feedstock, up close</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="n"/>
+      <c r="J26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n">
@@ -8363,7 +8389,7 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-17-worm-bin.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-17-aged-wood-chips.jpg</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
@@ -8373,7 +8399,7 @@
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>Photo 17 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 17 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -8383,21 +8409,21 @@
       </c>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>1200 x 1600</t>
+          <t>1600 x 1200</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>A wooden worm bin full of vermicompost under hanging lights</t>
+          <t>A pile of aged wood chips with a blue label reading "Aged wood chips"</t>
         </is>
       </c>
       <c r="H27" s="8" t="inlineStr">
         <is>
-          <t>The worm bin</t>
-        </is>
-      </c>
-      <c r="I27" s="8" t="inlineStr"/>
-      <c r="J27" s="8" t="inlineStr"/>
+          <t>Aged wood chips, ready for the pile</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
@@ -8405,7 +8431,7 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-18-microscopy-lab.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-18-alfalfa-cubes.jpg</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
@@ -8415,7 +8441,7 @@
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>Photo 18 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 18 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -8430,16 +8456,16 @@
       </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
-          <t>A microscopy lab: students at white microscopes and laptops while mentors point things out</t>
+          <t>A sack labeled "Alfalfa Cubes, net wt. 50 lb"</t>
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>The microscopy lab in full swing</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr"/>
-      <c r="J28" s="8" t="inlineStr"/>
+          <t>Alfalfa cubes for the compost recipe</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
@@ -8447,7 +8473,7 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-19-at-the-microscope.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-19-feedstock-buckets.jpg</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
@@ -8457,7 +8483,7 @@
       </c>
       <c r="D29" s="8" t="inlineStr">
         <is>
-          <t>Photo 19 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 19 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -8472,24 +8498,24 @@
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>A woman looking into a microscope, with a mentor in a plaid shirt behind her</t>
+          <t>Rows of blue buckets of dark feedstock, with a hoop house and a hill behind</t>
         </is>
       </c>
       <c r="H29" s="8" t="inlineStr">
         <is>
-          <t>Looking closely, with a mentor nearby</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr"/>
-      <c r="J29" s="8" t="inlineStr"/>
-    </row>
-    <row r="30">
+          <t>Feedstocks lined up for pile building</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="8" t="n"/>
+    </row>
+    <row r="30" ht="79.25" customHeight="1">
       <c r="A30" s="8" t="n">
         <v>26</v>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-20-mentor-with-microscopes.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-20-lifting-a-drum.jpg</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
@@ -8499,7 +8525,7 @@
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>Photo 20 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 20 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -8509,29 +8535,33 @@
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>1200 x 1600</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
-          <t>A white-bearded mentor smiling beside a row of microscopes</t>
+          <t>A man in a straw cowboy hat lifting a blue drum over a heap of feedstock beside a hoop house</t>
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>One of our mentors, all smiles at the microscopes</t>
-        </is>
-      </c>
-      <c r="I30" s="8" t="inlineStr"/>
-      <c r="J30" s="8" t="inlineStr"/>
-    </row>
-    <row r="31">
+          <t>Moving feedstock by the drum</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="79.25" customHeight="1">
       <c r="A31" s="8" t="n">
         <v>27</v>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-21-caps.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-21-carrying-a-drum.jpg</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
@@ -8541,7 +8571,7 @@
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>Photo 21 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 21 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -8551,29 +8581,33 @@
       </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>1600 x 900</t>
+          <t>1600 x 901</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>Dark green Soil Food Web caps on a table</t>
+          <t>A young man in a cap carrying a blue drum inside a hoop house, students and a pile of feedstock around him</t>
         </is>
       </c>
       <c r="H31" s="8" t="inlineStr">
         <is>
-          <t>Workshop caps, ready to wear</t>
-        </is>
-      </c>
-      <c r="I31" s="8" t="inlineStr"/>
-      <c r="J31" s="8" t="inlineStr"/>
-    </row>
-    <row r="32">
+          <t>Hauling drums in the hoop house</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="79.25" customHeight="1">
       <c r="A32" s="8" t="n">
         <v>28</v>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>accelerator-workshop-february-2026-gallery-22-certificate.jpg</t>
+          <t>accelerator-workshop-february-2026-gallery-22-everyone-in-close.jpg</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
@@ -8583,7 +8617,7 @@
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>Photo 22 of 22, under the heading "Photos from the workshop"</t>
+          <t>Photo 22 of 42, under the heading "Photos from the workshop"</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -8593,21 +8627,905 @@
       </c>
       <c r="F32" s="8" t="inlineStr">
         <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>The class crowded and crouching around blue buckets on the ground, seen from above</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>Everyone in close</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="79.25" customHeight="1">
+      <c r="A33" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-23-tiny-find.jpg</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Photo 23 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>An open palm with a tiny dark organism on it, close-up</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>A tiny find in the palm of a hand</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-24-thermometer-in-hay-bale.jpg</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Photo 24 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>A long-stem compost thermometer and a sun hat on a hay bale</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>The compost thermometer, always close at hand</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="n"/>
+      <c r="J34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-25-class-in-hoop-house.jpg</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Photo 25 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Students in caps and wide hats standing close together inside a hoop house, listening</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>Listening in the hoop house</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="n"/>
+      <c r="J35" s="8" t="n"/>
+    </row>
+    <row r="36" ht="79.25" customHeight="1">
+      <c r="A36" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-26-tossing-hay.jpg</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Photo 26 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>A man tossing hay onto a pile inside a hoop house, dust in the air</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>Building a pile in the hoop house</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="n"/>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="79.25" customHeight="1">
+      <c r="A37" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-27-lifting-the-cage.jpg</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Photo 27 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Two people lifting a wire cage off a compost pile inside a hoop house, a hay bale in front</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>Lifting the cage off a pile</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="n"/>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-28-insulated-compost-pile.jpg</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Photo 28 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>A woody compost pile in a hoop house, its base wrapped in reflective insulation</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>A pile wrapped up against the winter cold</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="n"/>
+      <c r="J38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-29-compost-row-in-hoop-house.jpg</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Photo 29 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>The inside of a hoop house with a long row of dark compost</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>A long row of compost in the hoop house</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="n"/>
+      <c r="J39" s="8" t="n"/>
+    </row>
+    <row r="40" ht="79.25" customHeight="1">
+      <c r="A40" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-30-checking-the-bin.jpg</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Photo 30 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>A woman in sunglasses kneeling at a wire compost bin and reaching into the pile, a blue bucket beside her</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Checking inside the bin</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="n"/>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="79.25" customHeight="1">
+      <c r="A41" s="8" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-31-smiles-at-the-bin.jpg</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Photo 31 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>A smiling woman in a purple hoodie and pink gloves leaning over a round wire bin, a man in a cap behind her</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>All smiles at the compost bin</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-32-worm-bin.jpg</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Photo 32 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>A wooden worm bin full of vermicompost under hanging lights</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>The worm bin</t>
+        </is>
+      </c>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-33-microscopy-lab.jpg</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Photo 33 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 1200</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>A microscopy lab: students at white microscopes and laptops while mentors point things out</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>The microscopy lab in full swing</t>
+        </is>
+      </c>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-34-at-the-microscope.jpg</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Photo 34 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
           <t>1600 x 900</t>
         </is>
       </c>
-      <c r="G32" s="8" t="inlineStr">
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>A woman looking into a microscope, with a mentor in a plaid shirt behind her</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>Looking closely, with a mentor nearby</t>
+        </is>
+      </c>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-35-mentor-with-microscopes.jpg</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Photo 35 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>1200 x 1600</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>A white-bearded mentor smiling beside a row of microscopes</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>One of our mentors, all smiles at the microscopes</t>
+        </is>
+      </c>
+      <c r="I45" s="8" t="n"/>
+      <c r="J45" s="8" t="n"/>
+    </row>
+    <row r="46" ht="79.25" customHeight="1">
+      <c r="A46" s="8" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-36-extraction-stands.jpg</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Photo 36 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>A man in a green shirt lifting a blue bucket beside white funnel stands with yellow tubing, students watching</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>At the extraction stands</t>
+        </is>
+      </c>
+      <c r="I46" s="8" t="n"/>
+      <c r="J46" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="79.25" customHeight="1">
+      <c r="A47" s="8" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-37-carts-by-the-dome.jpg</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Photo 37 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Students at rows of metal carts with equipment outdoors, a geodesic dome and bare trees behind</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>Working outdoors by the dome</t>
+        </is>
+      </c>
+      <c r="I47" s="8" t="n"/>
+      <c r="J47" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="79.25" customHeight="1">
+      <c r="A48" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-38-dinner-together.jpg</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Photo 38 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>The class around a long dinner table with plates of food, in a white room with paintings</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Dinner together</t>
+        </is>
+      </c>
+      <c r="I48" s="8" t="n"/>
+      <c r="J48" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="79.25" customHeight="1">
+      <c r="A49" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-39-birthday-candles.jpg</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Photo 39 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>A woman blowing out the candles on a chocolate birthday cake, a man standing beside her</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>Birthday candles</t>
+        </is>
+      </c>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="79.25" customHeight="1">
+      <c r="A50" s="8" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-40-sunset-over-the-mountains.jpg</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Photo 40 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 901</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Orange clouds over dark mountain silhouettes at sunset, scrub in the foreground</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Sunset over the mountains</t>
+        </is>
+      </c>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="inlineStr">
+        <is>
+          <t>Added 14 Oct 2026 (Photos-Feb26-CTPAW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-41-caps.jpg</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Photo 41 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 900</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>Dark green Soil Food Web caps on a table</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>Workshop caps, ready to wear</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="n"/>
+      <c r="J51" s="8" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>accelerator-workshop-february-2026-gallery-42-certificate.jpg</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>Gallery (bottom of page)</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Photo 42 of 42, under the heading "Photos from the workshop"</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>Justified grid of whole photos; click opens the full photo with its caption</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>1600 x 900</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
         <is>
           <t>Two people in an adobe room, one holding a graduation certificate</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr">
+      <c r="H52" s="8" t="inlineStr">
         <is>
           <t>A proud graduate</t>
         </is>
       </c>
-      <c r="I32" s="8" t="inlineStr"/>
-      <c r="J32" s="8" t="inlineStr"/>
+      <c r="I52" s="8" t="n"/>
+      <c r="J52" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>